<commit_message>
improve the excel processing
</commit_message>
<xml_diff>
--- a/src/output.xlsx
+++ b/src/output.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R44"/>
+  <dimension ref="A1:R45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -588,12 +588,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>: 30/01/2023</t>
+          <t>30/01/2023</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -634,12 +634,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>: 16/12/2022</t>
+          <t>16/12/2022</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -680,12 +680,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>: 08/11/2022</t>
+          <t>08/11/2022</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -726,12 +726,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>: 17/11/2022</t>
+          <t>17/11/2022</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -772,12 +772,12 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>: 29/05/2023</t>
+          <t>29/05/2023</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -819,12 +819,12 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>: 20/12/2022</t>
+          <t>20/12/2022</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -865,12 +865,12 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>: 06/01/2023</t>
+          <t>06/01/2023</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -912,12 +912,12 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>: 12/12/2022</t>
+          <t>12/12/2022</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -958,12 +958,12 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>: 30/01/2023</t>
+          <t>30/01/2023</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1006,12 +1006,12 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>: 12/12/2022</t>
+          <t>12/12/2022</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1053,12 +1053,12 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>: 30/01/2023</t>
+          <t>30/01/2023</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1099,12 +1099,12 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>: 05/12/2022</t>
+          <t>05/12/2022</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1145,12 +1145,12 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>: 15/03/2021</t>
+          <t>15/03/2021</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1191,12 +1191,12 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>: 14/07/2022</t>
+          <t>14/07/2022</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1237,12 +1237,12 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>: 09/01/2023</t>
+          <t>09/01/2023</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1283,12 +1283,12 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>: 20/12/2022</t>
+          <t>20/12/2022</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -1329,12 +1329,12 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>: 01/11/2022</t>
+          <t>01/11/2022</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -1375,12 +1375,12 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>: 20/12/2022</t>
+          <t>20/12/2022</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -1422,12 +1422,12 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>: 30/03/2022</t>
+          <t>30/03/2022</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -1468,12 +1468,12 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>: 01/11/2022</t>
+          <t>01/11/2022</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -1514,12 +1514,12 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>: 31/01/2023</t>
+          <t>31/01/2023</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -1561,12 +1561,12 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>: First Issued for Use</t>
+          <t>First Issued for Use</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -1608,12 +1608,12 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>: 27/06/2023</t>
+          <t>27/06/2023</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -1664,12 +1664,12 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>: 25/07/2022</t>
+          <t>25/07/2022</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -1720,12 +1720,12 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>: 29/06/2023</t>
+          <t>29/06/2023</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -1776,12 +1776,12 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>: 09/02/2022</t>
+          <t>09/02/2022</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -1831,12 +1831,12 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>: 30/01/2023</t>
+          <t>30/01/2023</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -1878,12 +1878,12 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>: 30/01/2023</t>
+          <t>30/01/2023</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -1923,12 +1923,12 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>: 26/08/2021</t>
+          <t>26/08/2021</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -1967,12 +1967,12 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>: First Issued for Use</t>
+          <t>First Issued for Use</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -2013,12 +2013,12 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>: First Issued for Use</t>
+          <t>First Issued for Use</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -2058,12 +2058,12 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>: First Issued for Use</t>
+          <t>First Issued for Use</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -2105,12 +2105,12 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>: First Issued for Use</t>
+          <t>First Issued for Use</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
@@ -2152,12 +2152,12 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>: First Issued for Use</t>
+          <t>First Issued for Use</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -2199,12 +2199,12 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>: First Issued for Use</t>
+          <t>First Issued for Use</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -2243,12 +2243,12 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>: First Issued for Use</t>
+          <t>First Issued for Use</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
@@ -2287,12 +2287,12 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>: First Issued for Use</t>
+          <t>First Issued for Use</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -2331,12 +2331,12 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>: First Issued for Use</t>
+          <t>First Issued for Use</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -2375,12 +2375,12 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>: First Issued for Use</t>
+          <t>First Issued for Use</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -2419,12 +2419,12 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>: First Issued for Use</t>
+          <t>First Issued for Use</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -2474,12 +2474,12 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>: First Issued for Use</t>
+          <t>First Issued for Use</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
@@ -2526,17 +2526,29 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>: First Issued for Use</t>
+          <t>First Issued for Use</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>: 01/04/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
           <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>tonne</t>
         </is>
       </c>
     </row>
@@ -2557,7 +2569,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Page No</t>
+          <t>No</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -2567,26 +2579,22 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Page1</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Error1</t>
+          <t>Testing error one</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Page2</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Error2</t>
+          <t>another testing error</t>
         </is>
       </c>
     </row>

</xml_diff>